<commit_message>
Added wildlife cameras to map
</commit_message>
<xml_diff>
--- a/Lokalitetarv2.xlsx
+++ b/Lokalitetarv2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nina-my.sharepoint.com/personal/christoffer_hilde_nina_no/Documents/Prosjekter/SEAPOP/Minkpredasjon/R/Lokaliteter/Minkprosjektet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="136" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCC2E9C6-0A40-4AEC-89FB-2011DF09262D}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{052E829B-3D7B-4D7A-A1E0-AC7DDAD1AC47}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="257">
   <si>
     <t xml:space="preserve">Forslag fra </t>
   </si>
@@ -432,9 +432,6 @@
     <t>Flakstad, Lofoten</t>
   </si>
   <si>
-    <t>Flakstadpollen, Flakstad, Øy ved Djupvika</t>
-  </si>
-  <si>
     <t>68.0749240049305, 13.338758227094258</t>
   </si>
   <si>
@@ -787,6 +784,21 @@
   </si>
   <si>
     <t>58.4817056, 8.9122654</t>
+  </si>
+  <si>
+    <t>Trond Vågsnes</t>
+  </si>
+  <si>
+    <t>Kristin Vågsnes/Rune Wærstad</t>
+  </si>
+  <si>
+    <t>951 18 979 / 906 35 765</t>
+  </si>
+  <si>
+    <t>Nøssfjord as</t>
+  </si>
+  <si>
+    <t>Flakstadpollen, Flakstad, Øy ved Djupvika (breinessteinan)</t>
   </si>
 </sst>
 </file>
@@ -1287,32 +1299,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V59"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="65" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="36" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="47.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="172.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="47.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="172.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1332,13 +1344,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>6</v>
@@ -1347,7 +1359,7 @@
         <v>7</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>8</v>
@@ -1380,7 +1392,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -1426,7 +1438,7 @@
       </c>
       <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1472,7 +1484,7 @@
       </c>
       <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>18</v>
       </c>
@@ -1518,7 +1530,7 @@
       </c>
       <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1564,7 +1576,7 @@
       </c>
       <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1610,7 +1622,7 @@
       </c>
       <c r="V6" s="4"/>
     </row>
-    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -1654,7 +1666,7 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1700,7 +1712,7 @@
       </c>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>18</v>
       </c>
@@ -1719,7 +1731,9 @@
       <c r="F9" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="26"/>
+      <c r="G9" s="26" t="s">
+        <v>61</v>
+      </c>
       <c r="H9" s="26"/>
       <c r="I9" s="26"/>
       <c r="J9" s="26" t="s">
@@ -1729,7 +1743,7 @@
         <v>25</v>
       </c>
       <c r="L9" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M9" s="26"/>
       <c r="N9" s="26" t="s">
@@ -1756,7 +1770,7 @@
       </c>
       <c r="V9" s="26"/>
     </row>
-    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>18</v>
       </c>
@@ -1785,7 +1799,7 @@
         <v>25</v>
       </c>
       <c r="L10" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M10" s="26"/>
       <c r="N10" s="26" t="s">
@@ -1812,7 +1826,7 @@
       </c>
       <c r="V10" s="26"/>
     </row>
-    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1831,7 +1845,9 @@
       <c r="F11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="5"/>
+      <c r="G11" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5" t="s">
@@ -1870,7 +1886,7 @@
       </c>
       <c r="V11" s="5"/>
     </row>
-    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
@@ -1928,7 +1944,7 @@
       </c>
       <c r="V12" s="5"/>
     </row>
-    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -1947,7 +1963,9 @@
       <c r="F13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="s">
@@ -1986,7 +2004,7 @@
       </c>
       <c r="V13" s="5"/>
     </row>
-    <row r="14" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -2044,7 +2062,7 @@
       </c>
       <c r="V14" s="5"/>
     </row>
-    <row r="15" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>18</v>
       </c>
@@ -2082,7 +2100,7 @@
       <c r="U15" s="9"/>
       <c r="V15" s="9"/>
     </row>
-    <row r="16" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>18</v>
       </c>
@@ -2120,7 +2138,7 @@
       <c r="U16" s="15"/>
       <c r="V16" s="15"/>
     </row>
-    <row r="17" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>18</v>
       </c>
@@ -2176,7 +2194,7 @@
       </c>
       <c r="V17" s="10"/>
     </row>
-    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>18</v>
       </c>
@@ -2228,7 +2246,7 @@
       <c r="U18" s="4"/>
       <c r="V18" s="4"/>
     </row>
-    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>18</v>
       </c>
@@ -2266,7 +2284,7 @@
       <c r="U19" s="9"/>
       <c r="V19" s="9"/>
     </row>
-    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>18</v>
       </c>
@@ -2304,7 +2322,7 @@
       <c r="U20" s="9"/>
       <c r="V20" s="9"/>
     </row>
-    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>18</v>
       </c>
@@ -2325,7 +2343,7 @@
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I21" s="10"/>
       <c r="J21" s="10" t="s">
@@ -2335,7 +2353,7 @@
         <v>72</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M21" s="10" t="s">
         <v>116</v>
@@ -2366,7 +2384,7 @@
       </c>
       <c r="V21" s="10"/>
     </row>
-    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -2390,7 +2408,7 @@
       <c r="U22" s="10"/>
       <c r="V22" s="10"/>
     </row>
-    <row r="23" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="28" t="s">
         <v>18</v>
       </c>
@@ -2417,7 +2435,7 @@
         <v>72</v>
       </c>
       <c r="L23" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M23" s="26"/>
       <c r="N23" s="26"/>
@@ -2430,7 +2448,7 @@
       <c r="U23" s="26"/>
       <c r="V23" s="26"/>
     </row>
-    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>18</v>
       </c>
@@ -2457,7 +2475,7 @@
         <v>72</v>
       </c>
       <c r="L24" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M24" s="26"/>
       <c r="N24" s="26"/>
@@ -2470,7 +2488,7 @@
       <c r="U24" s="26"/>
       <c r="V24" s="26"/>
     </row>
-    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="28" t="s">
         <v>18</v>
       </c>
@@ -2497,7 +2515,7 @@
         <v>72</v>
       </c>
       <c r="L25" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M25" s="26"/>
       <c r="N25" s="26"/>
@@ -2510,7 +2528,7 @@
       <c r="U25" s="26"/>
       <c r="V25" s="26"/>
     </row>
-    <row r="26" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>62</v>
       </c>
@@ -2518,13 +2536,13 @@
         <v>91</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F26" s="34" t="s">
         <v>23</v>
@@ -2533,11 +2551,11 @@
         <v>61</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>72</v>
@@ -2546,7 +2564,7 @@
         <v>61</v>
       </c>
       <c r="M26" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N26" s="10" t="s">
         <v>26</v>
@@ -2565,12 +2583,12 @@
         <v>62</v>
       </c>
       <c r="T26" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="U26" s="10"/>
       <c r="V26" s="10"/>
     </row>
-    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>18</v>
       </c>
@@ -2591,9 +2609,11 @@
       </c>
       <c r="G27" s="10"/>
       <c r="H27" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="I27" s="10"/>
+        <v>253</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>254</v>
+      </c>
       <c r="J27" s="10" t="s">
         <v>127</v>
       </c>
@@ -2632,7 +2652,7 @@
       </c>
       <c r="V27" s="10"/>
     </row>
-    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>18</v>
       </c>
@@ -2651,9 +2671,15 @@
       <c r="F28" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
+      <c r="G28" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="I28" s="7">
+        <v>41693935</v>
+      </c>
       <c r="J28" s="8"/>
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
@@ -2668,7 +2694,7 @@
       <c r="U28" s="9"/>
       <c r="V28" s="9"/>
     </row>
-    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>18</v>
       </c>
@@ -2679,19 +2705,25 @@
         <v>133</v>
       </c>
       <c r="D29" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
+      <c r="G29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="I29" s="5">
+        <v>97519210</v>
+      </c>
       <c r="J29" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K29" s="5" t="s">
         <v>72</v>
@@ -2716,7 +2748,7 @@
       <c r="U29" s="5"/>
       <c r="V29" s="5"/>
     </row>
-    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>18</v>
       </c>
@@ -2727,10 +2759,10 @@
         <v>133</v>
       </c>
       <c r="D30" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>138</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>23</v>
@@ -2739,7 +2771,7 @@
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>72</v>
@@ -2764,7 +2796,7 @@
       <c r="U30" s="5"/>
       <c r="V30" s="5"/>
     </row>
-    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>18</v>
       </c>
@@ -2775,10 +2807,10 @@
         <v>133</v>
       </c>
       <c r="D31" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>141</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>23</v>
@@ -2787,7 +2819,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>72</v>
@@ -2812,7 +2844,7 @@
       <c r="U31" s="5"/>
       <c r="V31" s="5"/>
     </row>
-    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>18</v>
       </c>
@@ -2823,10 +2855,10 @@
         <v>133</v>
       </c>
       <c r="D32" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E32" s="11" t="s">
         <v>143</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>144</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>23</v>
@@ -2835,7 +2867,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>72</v>
@@ -2860,7 +2892,7 @@
       <c r="U32" s="5"/>
       <c r="V32" s="5"/>
     </row>
-    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>18</v>
       </c>
@@ -2871,10 +2903,10 @@
         <v>133</v>
       </c>
       <c r="D33" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>146</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>147</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>23</v>
@@ -2883,7 +2915,7 @@
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>72</v>
@@ -2908,7 +2940,7 @@
       <c r="U33" s="4"/>
       <c r="V33" s="4"/>
     </row>
-    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>18</v>
       </c>
@@ -2919,10 +2951,10 @@
         <v>133</v>
       </c>
       <c r="D34" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="E34" s="12" t="s">
         <v>149</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>150</v>
       </c>
       <c r="F34" s="12" t="s">
         <v>23</v>
@@ -2931,7 +2963,7 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K34" s="12" t="s">
         <v>72</v>
@@ -2941,7 +2973,7 @@
       </c>
       <c r="M34" s="12"/>
       <c r="N34" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O34" s="12">
         <v>1</v>
@@ -2952,40 +2984,40 @@
       <c r="Q34" s="12"/>
       <c r="R34" s="12"/>
       <c r="S34" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T34" s="12" t="s">
         <v>75</v>
       </c>
       <c r="U34" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="V34" s="12"/>
+    </row>
+    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="V34" s="12"/>
-    </row>
-    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="4" t="s">
+      <c r="C35" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="E35" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K35" s="4" t="s">
         <v>72</v>
@@ -2994,10 +3026,10 @@
         <v>73</v>
       </c>
       <c r="M35" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="N35" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="N35" s="4" t="s">
-        <v>162</v>
       </c>
       <c r="O35" s="4">
         <v>0.2</v>
@@ -3016,34 +3048,34 @@
         <v>75</v>
       </c>
       <c r="U35" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="V35" s="4"/>
+    </row>
+    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D36" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="V35" s="4"/>
-    </row>
-    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="E36" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>165</v>
-      </c>
       <c r="F36" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>72</v>
@@ -3052,7 +3084,7 @@
         <v>73</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N36" s="4"/>
       <c r="O36" s="4">
@@ -3072,34 +3104,34 @@
         <v>75</v>
       </c>
       <c r="U36" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="D37" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>168</v>
-      </c>
       <c r="F37" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>72</v>
@@ -3108,10 +3140,10 @@
         <v>73</v>
       </c>
       <c r="M37" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N37" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O37" s="4">
         <v>0.2</v>
@@ -3130,34 +3162,34 @@
         <v>75</v>
       </c>
       <c r="U37" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="D38" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>72</v>
@@ -3166,10 +3198,10 @@
         <v>73</v>
       </c>
       <c r="M38" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="N38" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="N38" s="4" t="s">
-        <v>162</v>
       </c>
       <c r="O38" s="4">
         <v>0.2</v>
@@ -3188,34 +3220,34 @@
         <v>75</v>
       </c>
       <c r="U38" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="V38" s="4"/>
     </row>
-    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B39" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="C39" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="D39" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>72</v>
@@ -3224,10 +3256,10 @@
         <v>73</v>
       </c>
       <c r="M39" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O39" s="4">
         <v>0.2</v>
@@ -3246,11 +3278,11 @@
         <v>75</v>
       </c>
       <c r="U39" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="V39" s="4"/>
     </row>
-    <row r="40" spans="1:22" s="18" customFormat="1" ht="15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:22" s="18" customFormat="1" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
         <v>62</v>
       </c>
@@ -3258,22 +3290,22 @@
         <v>56</v>
       </c>
       <c r="C40" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D40" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="E40" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="F40" s="12" t="s">
         <v>180</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>181</v>
       </c>
       <c r="G40" s="12"/>
       <c r="H40" s="12"/>
       <c r="I40" s="12"/>
       <c r="J40" s="12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K40" s="12" t="s">
         <v>72</v>
@@ -3294,17 +3326,17 @@
       <c r="Q40" s="12"/>
       <c r="R40" s="12"/>
       <c r="S40" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T40" s="12" t="s">
         <v>128</v>
       </c>
       <c r="U40" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V40" s="12"/>
     </row>
-    <row r="41" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="36" t="s">
         <v>62</v>
       </c>
@@ -3312,20 +3344,20 @@
         <v>91</v>
       </c>
       <c r="C41" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="D41" s="36" t="s">
         <v>188</v>
-      </c>
-      <c r="D41" s="36" t="s">
-        <v>189</v>
       </c>
       <c r="E41" s="36"/>
       <c r="F41" s="36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G41" s="36"/>
       <c r="H41" s="36"/>
       <c r="I41" s="36"/>
       <c r="J41" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K41" s="12" t="s">
         <v>25</v>
@@ -3349,12 +3381,12 @@
         <v>62</v>
       </c>
       <c r="T41" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="U41" s="12"/>
       <c r="V41" s="12"/>
     </row>
-    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="36" t="s">
         <v>62</v>
       </c>
@@ -3362,10 +3394,10 @@
         <v>91</v>
       </c>
       <c r="C42" s="36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E42" s="36"/>
       <c r="F42" s="36" t="s">
@@ -3375,7 +3407,7 @@
       <c r="H42" s="36"/>
       <c r="I42" s="36"/>
       <c r="J42" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K42" s="12" t="s">
         <v>25</v>
@@ -3399,12 +3431,12 @@
         <v>62</v>
       </c>
       <c r="T42" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="U42" s="12"/>
       <c r="V42" s="12"/>
     </row>
-    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="36" t="s">
         <v>62</v>
       </c>
@@ -3412,10 +3444,10 @@
         <v>91</v>
       </c>
       <c r="C43" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="D43" s="36" t="s">
         <v>194</v>
-      </c>
-      <c r="D43" s="36" t="s">
-        <v>195</v>
       </c>
       <c r="E43" s="36"/>
       <c r="F43" s="36" t="s">
@@ -3425,7 +3457,7 @@
       <c r="H43" s="36"/>
       <c r="I43" s="36"/>
       <c r="J43" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K43" s="12" t="s">
         <v>25</v>
@@ -3449,26 +3481,26 @@
         <v>62</v>
       </c>
       <c r="T43" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="U43" s="12"/>
       <c r="V43" s="12"/>
     </row>
-    <row r="44" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C44" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D44" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="E44" s="10" t="s">
         <v>198</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>199</v>
       </c>
       <c r="F44" s="10" t="s">
         <v>61</v>
@@ -3477,7 +3509,7 @@
       <c r="H44" s="10"/>
       <c r="I44" s="10"/>
       <c r="J44" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K44" s="10" t="s">
         <v>25</v>
@@ -3486,10 +3518,10 @@
         <v>73</v>
       </c>
       <c r="M44" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N44" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O44" s="10">
         <v>1</v>
@@ -3505,27 +3537,27 @@
         <v>62</v>
       </c>
       <c r="T44" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="U44" s="10"/>
       <c r="V44" s="10"/>
     </row>
-    <row r="45" spans="1:22" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D45" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="E45" s="10" t="s">
-        <v>175</v>
-      </c>
       <c r="F45" s="10" t="s">
         <v>73</v>
       </c>
@@ -3533,13 +3565,13 @@
         <v>61</v>
       </c>
       <c r="H45" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I45" s="24">
         <v>48197464</v>
       </c>
       <c r="J45" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K45" s="10" t="s">
         <v>72</v>
@@ -3548,7 +3580,7 @@
         <v>61</v>
       </c>
       <c r="M45" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N45" s="10" t="s">
         <v>73</v>
@@ -3569,26 +3601,26 @@
         <v>62</v>
       </c>
       <c r="T45" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="U45" s="10"/>
       <c r="V45" s="10"/>
     </row>
-    <row r="46" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C46" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D46" s="34" t="s">
         <v>204</v>
       </c>
-      <c r="D46" s="34" t="s">
-        <v>205</v>
-      </c>
       <c r="E46" s="34" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F46" s="34" t="s">
         <v>73</v>
@@ -3597,7 +3629,7 @@
         <v>41</v>
       </c>
       <c r="H46" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I46" s="7"/>
       <c r="J46" s="8"/>
@@ -3618,21 +3650,21 @@
       <c r="U46" s="9"/>
       <c r="V46" s="9"/>
     </row>
-    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D47" s="35" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F47" s="34" t="s">
         <v>73</v>
@@ -3641,10 +3673,10 @@
         <v>61</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I47" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K47" s="10" t="s">
         <v>72</v>
@@ -3656,21 +3688,21 @@
         <v>73</v>
       </c>
     </row>
-    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D48" s="35" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E48" s="34" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F48" s="34" t="s">
         <v>61</v>
@@ -3679,7 +3711,7 @@
         <v>61</v>
       </c>
       <c r="H48" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I48" s="7">
         <v>91389435</v>
@@ -3688,27 +3720,27 @@
         <v>72</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="N48" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="49" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="26" t="s">
         <v>62</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C49" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="D49" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="D49" s="27" t="s">
-        <v>209</v>
-      </c>
       <c r="E49" s="26" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F49" s="28" t="s">
         <v>61</v>
@@ -3717,7 +3749,7 @@
         <v>61</v>
       </c>
       <c r="H49" s="28" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I49" s="28">
         <v>94123558</v>
@@ -3726,27 +3758,27 @@
         <v>25</v>
       </c>
       <c r="L49" s="27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="N49" s="26" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="26" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C50" s="26" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D50" s="27" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E50" s="26" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F50" s="28" t="s">
         <v>61</v>
@@ -3760,27 +3792,27 @@
         <v>25</v>
       </c>
       <c r="L50" s="27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="N50" s="26" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D51" s="35" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E51" s="35" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F51" s="34" t="s">
         <v>61</v>
@@ -3789,10 +3821,10 @@
         <v>61</v>
       </c>
       <c r="H51" t="s">
+        <v>245</v>
+      </c>
+      <c r="I51" t="s">
         <v>246</v>
-      </c>
-      <c r="I51" t="s">
-        <v>247</v>
       </c>
       <c r="K51" s="10" t="s">
         <v>72</v>
@@ -3804,21 +3836,21 @@
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>62</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F52" s="34" t="s">
         <v>73</v>
@@ -3838,7 +3870,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="53" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="26" t="s">
         <v>18</v>
       </c>
@@ -3846,10 +3878,10 @@
         <v>56</v>
       </c>
       <c r="D53" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="E53" s="29" t="s">
         <v>221</v>
-      </c>
-      <c r="E53" s="29" t="s">
-        <v>222</v>
       </c>
       <c r="F53" s="31" t="s">
         <v>61</v>
@@ -3861,10 +3893,10 @@
         <v>25</v>
       </c>
       <c r="L53" s="30" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>18</v>
       </c>
@@ -3872,10 +3904,10 @@
         <v>56</v>
       </c>
       <c r="D54" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="E54" t="s">
         <v>223</v>
-      </c>
-      <c r="E54" t="s">
-        <v>224</v>
       </c>
       <c r="F54" s="21" t="s">
         <v>61</v>
@@ -3890,7 +3922,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>18</v>
       </c>
@@ -3898,7 +3930,7 @@
         <v>56</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="K55" s="20" t="s">
         <v>72</v>
@@ -3907,7 +3939,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>18</v>
       </c>
@@ -3915,13 +3947,13 @@
         <v>56</v>
       </c>
       <c r="C56" t="s">
+        <v>226</v>
+      </c>
+      <c r="D56" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="E56" t="s">
         <v>227</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="E56" t="s">
-        <v>228</v>
       </c>
       <c r="K56" s="20" t="s">
         <v>72</v>
@@ -3930,7 +3962,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>18</v>
       </c>
@@ -3938,13 +3970,13 @@
         <v>56</v>
       </c>
       <c r="C57" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D57" t="s">
+        <v>228</v>
+      </c>
+      <c r="E57" t="s">
         <v>229</v>
-      </c>
-      <c r="E57" t="s">
-        <v>230</v>
       </c>
       <c r="K57" s="20" t="s">
         <v>72</v>
@@ -3953,7 +3985,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>18</v>
       </c>
@@ -3961,22 +3993,22 @@
         <v>56</v>
       </c>
       <c r="C58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D58" t="s">
+        <v>231</v>
+      </c>
+      <c r="E58" t="s">
         <v>232</v>
-      </c>
-      <c r="E58" t="s">
-        <v>233</v>
       </c>
       <c r="K58" s="20" t="s">
         <v>72</v>
       </c>
       <c r="L58" s="19" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>18</v>
       </c>
@@ -3984,13 +4016,13 @@
         <v>56</v>
       </c>
       <c r="C59" t="s">
+        <v>234</v>
+      </c>
+      <c r="D59" t="s">
         <v>235</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>236</v>
-      </c>
-      <c r="E59" t="s">
-        <v>237</v>
       </c>
       <c r="F59" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
Lagt til Nordre Steinskjæret, fjerna Tjeldstø
</commit_message>
<xml_diff>
--- a/Lokalitetarv2.xlsx
+++ b/Lokalitetarv2.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nina-my.sharepoint.com/personal/christoffer_hilde_nina_no/Documents/Prosjekter/SEAPOP/Minkpredasjon/R/Lokaliteter/Minkprosjektet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{052E829B-3D7B-4D7A-A1E0-AC7DDAD1AC47}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A975233-21C3-43C5-9B7C-C2AE2BDB318F}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$V$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$V$60</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="259">
   <si>
     <t xml:space="preserve">Forslag fra </t>
   </si>
@@ -799,6 +799,12 @@
   </si>
   <si>
     <t>Flakstadpollen, Flakstad, Øy ved Djupvika (breinessteinan)</t>
+  </si>
+  <si>
+    <t>Nordre Steinskjæret</t>
+  </si>
+  <si>
+    <t>60.268689000296455, 5.219000199094522</t>
   </si>
 </sst>
 </file>
@@ -1298,33 +1304,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:V60"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="65" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="36" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="172.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="47.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="172.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1392,7 +1398,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -1438,7 +1444,7 @@
       </c>
       <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1484,7 +1490,7 @@
       </c>
       <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>18</v>
       </c>
@@ -1530,7 +1536,7 @@
       </c>
       <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1576,7 +1582,7 @@
       </c>
       <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1622,7 +1628,7 @@
       </c>
       <c r="V6" s="4"/>
     </row>
-    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -1666,7 +1672,7 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1712,7 +1718,7 @@
       </c>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>18</v>
       </c>
@@ -1770,7 +1776,7 @@
       </c>
       <c r="V9" s="26"/>
     </row>
-    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>18</v>
       </c>
@@ -1826,7 +1832,7 @@
       </c>
       <c r="V10" s="26"/>
     </row>
-    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1886,7 +1892,7 @@
       </c>
       <c r="V11" s="5"/>
     </row>
-    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
@@ -1944,7 +1950,7 @@
       </c>
       <c r="V12" s="5"/>
     </row>
-    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -2004,287 +2010,291 @@
       </c>
       <c r="V13" s="5"/>
     </row>
-    <row r="14" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="5" t="s">
+    <row r="14" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5" t="s">
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="O14" s="5">
+      <c r="L14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="O14" s="12">
         <v>2</v>
       </c>
-      <c r="P14" s="5">
+      <c r="P14" s="12">
         <v>5</v>
       </c>
-      <c r="Q14" s="5">
+      <c r="Q14" s="12">
         <v>2</v>
       </c>
-      <c r="R14" s="5" t="s">
+      <c r="R14" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="S14" s="5" t="s">
+      <c r="S14" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="T14" s="5" t="s">
+      <c r="T14" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="U14" s="5" t="s">
+      <c r="U14" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="V14" s="5"/>
-    </row>
-    <row r="15" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="7" t="s">
+      <c r="V14" s="12"/>
+    </row>
+    <row r="15" spans="1:22" s="35" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+    </row>
+    <row r="16" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C16" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-    </row>
-    <row r="16" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="14" t="s">
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9"/>
+      <c r="U16" s="9"/>
+      <c r="V16" s="9"/>
+    </row>
+    <row r="17" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C17" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F17" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15"/>
-    </row>
-    <row r="17" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+      <c r="V17" s="15"/>
+    </row>
+    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C18" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E18" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10" t="s">
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="K17" s="10" t="s">
+      <c r="K18" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L17" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="L18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="N17" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="O17" s="10">
+      <c r="N18" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="O18" s="10">
         <v>1</v>
       </c>
-      <c r="P17" s="10">
+      <c r="P18" s="10">
         <v>1</v>
       </c>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="10" t="s">
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="T17" s="10" t="s">
+      <c r="T18" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="U17" s="10" t="s">
+      <c r="U18" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="V17" s="10"/>
-    </row>
-    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="V18" s="10"/>
+    </row>
+    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4" t="s">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4" t="s">
+      <c r="L19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O18" s="4">
+      <c r="O19" s="4">
         <v>1</v>
       </c>
-      <c r="P18" s="4">
+      <c r="P19" s="4">
         <v>1</v>
       </c>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="4" t="s">
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="T18" s="4" t="s">
+      <c r="T19" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="U18" s="4"/>
-      <c r="V18" s="4"/>
-    </row>
-    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
-      <c r="S19" s="9"/>
-      <c r="T19" s="9"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9"/>
-    </row>
-    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+    </row>
+    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>18</v>
       </c>
@@ -2295,10 +2305,10 @@
         <v>107</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>23</v>
@@ -2322,133 +2332,131 @@
       <c r="U20" s="9"/>
       <c r="V20" s="9"/>
     </row>
-    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="10" t="s">
+    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+    </row>
+    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D22" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F22" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10" t="s">
+      <c r="G22" s="10"/>
+      <c r="H22" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10" t="s">
+      <c r="I22" s="10"/>
+      <c r="J22" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K22" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L22" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="M21" s="10" t="s">
+      <c r="M22" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="N21" s="10" t="s">
+      <c r="N22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O21" s="10">
+      <c r="O22" s="10">
         <v>2</v>
       </c>
-      <c r="P21" s="10">
+      <c r="P22" s="10">
         <v>1</v>
       </c>
-      <c r="Q21" s="10">
+      <c r="Q22" s="10">
         <v>2</v>
       </c>
-      <c r="R21" s="10" t="s">
+      <c r="R22" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="S21" s="10" t="s">
+      <c r="S22" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="T21" s="10" t="s">
+      <c r="T22" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="U21" s="10" t="s">
+      <c r="U22" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="V21" s="10"/>
-    </row>
-    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
-      <c r="R22" s="10"/>
-      <c r="S22" s="10"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="10"/>
       <c r="V22" s="10"/>
     </row>
-    <row r="23" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="E23" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="F23" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="L23" s="26" t="s">
-        <v>202</v>
-      </c>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="26"/>
-      <c r="R23" s="26"/>
-      <c r="S23" s="26"/>
-      <c r="T23" s="26"/>
-      <c r="U23" s="26"/>
-      <c r="V23" s="26"/>
-    </row>
-    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10"/>
+    </row>
+    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="28" t="s">
         <v>18</v>
       </c>
@@ -2459,10 +2467,10 @@
         <v>112</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F24" s="28" t="s">
         <v>23</v>
@@ -2488,7 +2496,7 @@
       <c r="U24" s="26"/>
       <c r="V24" s="26"/>
     </row>
-    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="28" t="s">
         <v>18</v>
       </c>
@@ -2499,10 +2507,10 @@
         <v>112</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F25" s="28" t="s">
         <v>23</v>
@@ -2528,94 +2536,74 @@
       <c r="U25" s="26"/>
       <c r="V25" s="26"/>
     </row>
-    <row r="26" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="L26" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
+      <c r="Q26" s="26"/>
+      <c r="R26" s="26"/>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="26"/>
+      <c r="V26" s="26"/>
+    </row>
+    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="F26" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="K26" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="L26" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="M26" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="N26" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O26" s="10">
-        <v>1</v>
-      </c>
-      <c r="P26" s="10">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="10">
-        <v>1</v>
-      </c>
-      <c r="R26" s="10"/>
-      <c r="S26" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="T26" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10"/>
-    </row>
-    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>91</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>124</v>
+        <v>183</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>125</v>
+        <v>249</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="10" t="s">
+        <v>251</v>
+      </c>
+      <c r="F27" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10" t="s">
+        <v>61</v>
+      </c>
       <c r="H27" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>254</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="I27" s="10"/>
       <c r="J27" s="10" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>72</v>
@@ -2624,10 +2612,10 @@
         <v>61</v>
       </c>
       <c r="M27" s="10" t="s">
-        <v>116</v>
+        <v>185</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="O27" s="10">
         <v>1</v>
@@ -2636,119 +2624,125 @@
         <v>1</v>
       </c>
       <c r="Q27" s="10">
-        <v>2</v>
-      </c>
-      <c r="R27" s="10" t="s">
-        <v>81</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R27" s="10"/>
       <c r="S27" s="10" t="s">
         <v>62</v>
       </c>
       <c r="T27" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10"/>
+    </row>
+    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L28" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M28" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="N28" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="O28" s="10">
+        <v>1</v>
+      </c>
+      <c r="P28" s="10">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="10">
+        <v>2</v>
+      </c>
+      <c r="R28" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="S28" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="T28" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="U27" s="13" t="s">
+      <c r="U28" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="V27" s="10"/>
-    </row>
-    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="V28" s="10"/>
+    </row>
+    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C29" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F29" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H28" s="7" t="s">
+      <c r="G29" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="I28" s="7">
+      <c r="I29" s="7">
         <v>41693935</v>
       </c>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
-      <c r="S28" s="9"/>
-      <c r="T28" s="9"/>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9"/>
-    </row>
-    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="I29" s="5">
-        <v>97519210</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="L29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O29" s="5">
-        <v>1</v>
-      </c>
-      <c r="P29" s="5">
-        <v>2</v>
-      </c>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="5"/>
-    </row>
-    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J29" s="8"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="9"/>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
+      <c r="S29" s="9"/>
+      <c r="T29" s="9"/>
+      <c r="U29" s="9"/>
+      <c r="V29" s="9"/>
+    </row>
+    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>18</v>
       </c>
@@ -2759,19 +2753,25 @@
         <v>133</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>136</v>
+        <v>256</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="G30" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="I30" s="5">
+        <v>97519210</v>
+      </c>
       <c r="J30" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>72</v>
@@ -2796,7 +2796,7 @@
       <c r="U30" s="5"/>
       <c r="V30" s="5"/>
     </row>
-    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>18</v>
       </c>
@@ -2807,10 +2807,10 @@
         <v>133</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>23</v>
@@ -2819,7 +2819,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>72</v>
@@ -2844,7 +2844,7 @@
       <c r="U31" s="5"/>
       <c r="V31" s="5"/>
     </row>
-    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>18</v>
       </c>
@@ -2855,10 +2855,10 @@
         <v>133</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>143</v>
+        <v>139</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>23</v>
@@ -2867,7 +2867,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>72</v>
@@ -2892,167 +2892,157 @@
       <c r="U32" s="5"/>
       <c r="V32" s="5"/>
     </row>
-    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" s="4" t="s">
+    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="O33" s="5">
+        <v>1</v>
+      </c>
+      <c r="P33" s="5">
+        <v>2</v>
+      </c>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="5"/>
+    </row>
+    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E34" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4" t="s">
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="K33" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="L33" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4" t="s">
+      <c r="L34" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O34" s="4">
         <v>1</v>
       </c>
-      <c r="P33" s="4">
+      <c r="P34" s="4">
         <v>2</v>
       </c>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="4"/>
-      <c r="T33" s="4"/>
-      <c r="U33" s="4"/>
-      <c r="V33" s="4"/>
-    </row>
-    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="12" t="s">
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
+      <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="4"/>
+      <c r="V34" s="4"/>
+    </row>
+    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C35" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D35" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E35" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="F34" s="12" t="s">
+      <c r="F35" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12" t="s">
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="K34" s="12" t="s">
+      <c r="K35" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="L34" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12" t="s">
+      <c r="L35" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="O34" s="12">
+      <c r="O35" s="12">
         <v>1</v>
       </c>
-      <c r="P34" s="12">
+      <c r="P35" s="12">
         <v>4</v>
       </c>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="12" t="s">
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="T34" s="12" t="s">
+      <c r="T35" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="U34" s="12" t="s">
+      <c r="U35" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="V34" s="12"/>
-    </row>
-    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="L35" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M35" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="N35" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="O35" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="P35" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="Q35" s="4">
-        <v>1</v>
-      </c>
-      <c r="R35" s="4"/>
-      <c r="S35" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="T35" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="U35" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="V35" s="4"/>
-    </row>
-    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="V35" s="12"/>
+    </row>
+    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>18</v>
       </c>
@@ -3063,10 +3053,10 @@
         <v>155</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>158</v>
@@ -3075,7 +3065,7 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>72</v>
@@ -3086,7 +3076,9 @@
       <c r="M36" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="N36" s="4"/>
+      <c r="N36" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="O36" s="4">
         <v>0.2</v>
       </c>
@@ -3108,7 +3100,7 @@
       </c>
       <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>18</v>
       </c>
@@ -3119,10 +3111,10 @@
         <v>155</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>158</v>
@@ -3131,7 +3123,7 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>72</v>
@@ -3142,9 +3134,7 @@
       <c r="M37" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="N37" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="N37" s="4"/>
       <c r="O37" s="4">
         <v>0.2</v>
       </c>
@@ -3166,7 +3156,7 @@
       </c>
       <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>18</v>
       </c>
@@ -3177,7 +3167,7 @@
         <v>155</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>167</v>
@@ -3189,7 +3179,7 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>72</v>
@@ -3201,7 +3191,7 @@
         <v>160</v>
       </c>
       <c r="N38" s="4" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="O38" s="4">
         <v>0.2</v>
@@ -3224,7 +3214,7 @@
       </c>
       <c r="V38" s="4"/>
     </row>
-    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>18</v>
       </c>
@@ -3235,7 +3225,7 @@
         <v>155</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>167</v>
@@ -3247,7 +3237,7 @@
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>72</v>
@@ -3259,7 +3249,7 @@
         <v>160</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="O39" s="4">
         <v>0.2</v>
@@ -3268,7 +3258,7 @@
         <v>0.5</v>
       </c>
       <c r="Q39" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R39" s="4"/>
       <c r="S39" s="4" t="s">
@@ -3278,96 +3268,102 @@
         <v>75</v>
       </c>
       <c r="U39" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="V39" s="4"/>
+    </row>
+    <row r="40" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L40" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="O40" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="P40" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>2</v>
+      </c>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="T40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="U40" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="V39" s="4"/>
-    </row>
-    <row r="40" spans="1:22" s="18" customFormat="1" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="V40" s="4"/>
+    </row>
+    <row r="41" spans="1:22" s="18" customFormat="1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C41" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D41" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E41" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="F41" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12" t="s">
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="K40" s="12" t="s">
+      <c r="K41" s="12" t="s">
         <v>72</v>
-      </c>
-      <c r="L40" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="M40" s="12"/>
-      <c r="N40" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="O40" s="12">
-        <v>1</v>
-      </c>
-      <c r="P40" s="12">
-        <v>1</v>
-      </c>
-      <c r="Q40" s="12"/>
-      <c r="R40" s="12"/>
-      <c r="S40" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="T40" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="U40" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="V40" s="12"/>
-    </row>
-    <row r="41" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="36" t="s">
-        <v>62</v>
-      </c>
-      <c r="B41" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="C41" s="36" t="s">
-        <v>187</v>
-      </c>
-      <c r="D41" s="36" t="s">
-        <v>188</v>
-      </c>
-      <c r="E41" s="36"/>
-      <c r="F41" s="36" t="s">
-        <v>189</v>
-      </c>
-      <c r="G41" s="36"/>
-      <c r="H41" s="36"/>
-      <c r="I41" s="36"/>
-      <c r="J41" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="K41" s="12" t="s">
-        <v>25</v>
       </c>
       <c r="L41" s="12" t="s">
         <v>73</v>
       </c>
       <c r="M41" s="12"/>
       <c r="N41" s="12" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="O41" s="12">
         <v>1</v>
@@ -3378,15 +3374,17 @@
       <c r="Q41" s="12"/>
       <c r="R41" s="12"/>
       <c r="S41" s="12" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
       <c r="T41" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="U41" s="12"/>
+        <v>128</v>
+      </c>
+      <c r="U41" s="12" t="s">
+        <v>182</v>
+      </c>
       <c r="V41" s="12"/>
     </row>
-    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="36" t="s">
         <v>62</v>
       </c>
@@ -3397,17 +3395,17 @@
         <v>187</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E42" s="36"/>
       <c r="F42" s="36" t="s">
-        <v>73</v>
+        <v>189</v>
       </c>
       <c r="G42" s="36"/>
       <c r="H42" s="36"/>
       <c r="I42" s="36"/>
       <c r="J42" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K42" s="12" t="s">
         <v>25</v>
@@ -3417,7 +3415,7 @@
       </c>
       <c r="M42" s="12"/>
       <c r="N42" s="12" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="O42" s="12">
         <v>1</v>
@@ -3436,7 +3434,7 @@
       <c r="U42" s="12"/>
       <c r="V42" s="12"/>
     </row>
-    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="36" t="s">
         <v>62</v>
       </c>
@@ -3444,10 +3442,10 @@
         <v>91</v>
       </c>
       <c r="C43" s="36" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D43" s="36" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E43" s="36"/>
       <c r="F43" s="36" t="s">
@@ -3457,7 +3455,7 @@
       <c r="H43" s="36"/>
       <c r="I43" s="36"/>
       <c r="J43" s="12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K43" s="12" t="s">
         <v>25</v>
@@ -3467,7 +3465,7 @@
       </c>
       <c r="M43" s="12"/>
       <c r="N43" s="12" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="O43" s="12">
         <v>1</v>
@@ -3486,63 +3484,57 @@
       <c r="U43" s="12"/>
       <c r="V43" s="12"/>
     </row>
-    <row r="44" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B44" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="K44" s="10" t="s">
+      <c r="B44" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="D44" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
+      <c r="J44" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="K44" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="L44" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="M44" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="N44" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="O44" s="10">
+      <c r="L44" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M44" s="12"/>
+      <c r="N44" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="O44" s="12">
         <v>1</v>
       </c>
-      <c r="P44" s="10">
+      <c r="P44" s="12">
         <v>1</v>
       </c>
-      <c r="Q44" s="10">
-        <v>3</v>
-      </c>
-      <c r="R44" s="10"/>
-      <c r="S44" s="10" t="s">
+      <c r="Q44" s="12"/>
+      <c r="R44" s="12"/>
+      <c r="S44" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="T44" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="U44" s="10"/>
-      <c r="V44" s="10"/>
-    </row>
-    <row r="45" spans="1:22" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T44" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="U44" s="12"/>
+      <c r="V44" s="12"/>
+    </row>
+    <row r="45" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="s">
         <v>62</v>
       </c>
@@ -3550,63 +3542,55 @@
         <v>154</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G45" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="H45" t="s">
-        <v>242</v>
-      </c>
-      <c r="I45" s="24">
-        <v>48197464</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
       <c r="J45" s="10" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="M45" s="10" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>73</v>
+        <v>161</v>
       </c>
       <c r="O45" s="10">
         <v>1</v>
       </c>
       <c r="P45" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q45" s="10">
-        <v>4</v>
-      </c>
-      <c r="R45" s="10">
-        <v>2</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R45" s="10"/>
       <c r="S45" s="10" t="s">
         <v>62</v>
       </c>
       <c r="T45" s="10" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="U45" s="10"/>
       <c r="V45" s="10"/>
     </row>
-    <row r="46" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>62</v>
       </c>
@@ -3616,41 +3600,61 @@
       <c r="C46" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D46" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="E46" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="F46" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="G46" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="I46" s="7"/>
-      <c r="J46" s="8"/>
+      <c r="D46" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G46" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="H46" t="s">
+        <v>242</v>
+      </c>
+      <c r="I46" s="24">
+        <v>48197464</v>
+      </c>
+      <c r="J46" s="10" t="s">
+        <v>175</v>
+      </c>
       <c r="K46" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L46" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="M46" s="9"/>
-      <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="9"/>
-      <c r="Q46" s="9"/>
-      <c r="R46" s="9"/>
-      <c r="S46" s="9"/>
-      <c r="T46" s="9"/>
-      <c r="U46" s="9"/>
-      <c r="V46" s="9"/>
-    </row>
-    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L46" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M46" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="N46" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="O46" s="10">
+        <v>1</v>
+      </c>
+      <c r="P46" s="10">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="10">
+        <v>4</v>
+      </c>
+      <c r="R46" s="10">
+        <v>2</v>
+      </c>
+      <c r="S46" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="T46" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="U46" s="10"/>
+      <c r="V46" s="10"/>
+    </row>
+    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>62</v>
       </c>
@@ -3660,35 +3664,41 @@
       <c r="C47" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D47" s="35" t="s">
-        <v>205</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>216</v>
+      <c r="D47" s="34" t="s">
+        <v>204</v>
+      </c>
+      <c r="E47" s="34" t="s">
+        <v>217</v>
       </c>
       <c r="F47" s="34" t="s">
         <v>73</v>
       </c>
       <c r="G47" s="34" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>243</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="I47" s="7"/>
+      <c r="J47" s="8"/>
       <c r="K47" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L47" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="N47" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L47" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="9"/>
+      <c r="R47" s="9"/>
+      <c r="S47" s="9"/>
+      <c r="T47" s="9"/>
+      <c r="U47" s="9"/>
+      <c r="V47" s="9"/>
+    </row>
+    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>62</v>
       </c>
@@ -3699,72 +3709,72 @@
         <v>203</v>
       </c>
       <c r="D48" s="35" t="s">
-        <v>206</v>
-      </c>
-      <c r="E48" s="34" t="s">
-        <v>218</v>
+        <v>205</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>216</v>
       </c>
       <c r="F48" s="34" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="G48" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="H48" t="s">
-        <v>247</v>
-      </c>
-      <c r="I48" s="7">
-        <v>91389435</v>
+      <c r="H48" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="I48" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="K48" s="10" t="s">
         <v>72</v>
       </c>
       <c r="L48" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N48" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D49" s="35" t="s">
+        <v>206</v>
+      </c>
+      <c r="E49" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="F49" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="G49" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="H49" t="s">
+        <v>247</v>
+      </c>
+      <c r="I49" s="7">
+        <v>91389435</v>
+      </c>
+      <c r="K49" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L49" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="N48" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="B49" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>207</v>
-      </c>
-      <c r="D49" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="E49" s="26" t="s">
-        <v>215</v>
-      </c>
-      <c r="F49" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="G49" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="H49" s="28" t="s">
-        <v>240</v>
-      </c>
-      <c r="I49" s="28">
-        <v>94123558</v>
-      </c>
-      <c r="K49" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="L49" s="27" t="s">
-        <v>202</v>
-      </c>
-      <c r="N49" s="26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N49" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="26" t="s">
         <v>62</v>
       </c>
@@ -3775,10 +3785,10 @@
         <v>207</v>
       </c>
       <c r="D50" s="27" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E50" s="26" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F50" s="28" t="s">
         <v>61</v>
@@ -3786,8 +3796,12 @@
       <c r="G50" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="H50" s="28"/>
-      <c r="I50" s="28"/>
+      <c r="H50" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="I50" s="28">
+        <v>94123558</v>
+      </c>
       <c r="K50" s="26" t="s">
         <v>25</v>
       </c>
@@ -3798,45 +3812,41 @@
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10" t="s">
+    <row r="51" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B51" s="10" t="s">
+      <c r="B51" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="D51" s="35" t="s">
-        <v>209</v>
-      </c>
-      <c r="E51" s="35" t="s">
-        <v>211</v>
-      </c>
-      <c r="F51" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="G51" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="H51" t="s">
-        <v>245</v>
-      </c>
-      <c r="I51" t="s">
-        <v>246</v>
-      </c>
-      <c r="K51" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="N51" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D51" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="E51" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="F51" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="G51" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="H51" s="28"/>
+      <c r="I51" s="28"/>
+      <c r="K51" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="L51" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="N51" s="26" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
         <v>62</v>
       </c>
@@ -3847,19 +3857,23 @@
         <v>207</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>212</v>
+        <v>209</v>
+      </c>
+      <c r="E52" s="35" t="s">
+        <v>211</v>
       </c>
       <c r="F52" s="34" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="G52" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
+        <v>61</v>
+      </c>
+      <c r="H52" t="s">
+        <v>245</v>
+      </c>
+      <c r="I52" t="s">
+        <v>246</v>
+      </c>
       <c r="K52" s="10" t="s">
         <v>72</v>
       </c>
@@ -3870,59 +3884,67 @@
         <v>73</v>
       </c>
     </row>
-    <row r="53" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="B53" s="26" t="s">
+    <row r="53" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D53" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="F53" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="G53" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="K53" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N53" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D53" s="30" t="s">
+      <c r="D54" s="30" t="s">
         <v>220</v>
       </c>
-      <c r="E53" s="29" t="s">
+      <c r="E54" s="29" t="s">
         <v>221</v>
       </c>
-      <c r="F53" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="G53" s="32"/>
-      <c r="H53" s="32"/>
-      <c r="I53" s="32"/>
-      <c r="K53" s="33" t="s">
+      <c r="F54" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="G54" s="32"/>
+      <c r="H54" s="32"/>
+      <c r="I54" s="32"/>
+      <c r="K54" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="L53" s="30" t="s">
+      <c r="L54" s="30" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="E54" t="s">
-        <v>223</v>
-      </c>
-      <c r="F54" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="K54" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="L54" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>18</v>
       </c>
@@ -3930,8 +3952,17 @@
         <v>56</v>
       </c>
       <c r="D55" s="19" t="s">
-        <v>224</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="E55" t="s">
+        <v>223</v>
+      </c>
+      <c r="F55" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G55" s="23"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
       <c r="K55" s="20" t="s">
         <v>72</v>
       </c>
@@ -3939,30 +3970,24 @@
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C56" t="s">
-        <v>226</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="E56" t="s">
-        <v>227</v>
+      <c r="D56" s="19" t="s">
+        <v>224</v>
       </c>
       <c r="K56" s="20" t="s">
         <v>72</v>
       </c>
       <c r="L56" s="19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>18</v>
       </c>
@@ -3970,22 +3995,22 @@
         <v>56</v>
       </c>
       <c r="C57" t="s">
-        <v>230</v>
-      </c>
-      <c r="D57" t="s">
-        <v>228</v>
+        <v>226</v>
+      </c>
+      <c r="D57" s="22" t="s">
+        <v>225</v>
       </c>
       <c r="E57" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="K57" s="20" t="s">
         <v>72</v>
       </c>
       <c r="L57" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>18</v>
       </c>
@@ -3993,13 +4018,13 @@
         <v>56</v>
       </c>
       <c r="C58" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D58" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E58" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="K58" s="20" t="s">
         <v>72</v>
@@ -4008,7 +4033,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>18</v>
       </c>
@@ -4016,16 +4041,13 @@
         <v>56</v>
       </c>
       <c r="C59" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D59" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E59" t="s">
-        <v>236</v>
-      </c>
-      <c r="F59" t="s">
-        <v>73</v>
+        <v>232</v>
       </c>
       <c r="K59" s="20" t="s">
         <v>72</v>
@@ -4034,8 +4056,34 @@
         <v>61</v>
       </c>
     </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60" t="s">
+        <v>234</v>
+      </c>
+      <c r="D60" t="s">
+        <v>235</v>
+      </c>
+      <c r="E60" t="s">
+        <v>236</v>
+      </c>
+      <c r="F60" t="s">
+        <v>73</v>
+      </c>
+      <c r="K60" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="L60" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V59" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V60" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Lagt til Nordre Steinskjæret, fjerna Tjeldstø. Fiksa lokalitetsnamn,
</commit_message>
<xml_diff>
--- a/Lokalitetarv2.xlsx
+++ b/Lokalitetarv2.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nina-my.sharepoint.com/personal/christoffer_hilde_nina_no/Documents/Prosjekter/SEAPOP/Minkpredasjon/R/Lokaliteter/Minkprosjektet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{052E829B-3D7B-4D7A-A1E0-AC7DDAD1AC47}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{D4F2DE48-26F6-417C-88E3-7EC1ECC2050D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEC5ADF5-C422-4D1B-9E1A-C089D8E1FEF1}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$V$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ark1'!$A$1:$V$60</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="260">
   <si>
     <t xml:space="preserve">Forslag fra </t>
   </si>
@@ -732,9 +732,6 @@
     <t>Alvøen</t>
   </si>
   <si>
-    <t>Espeland</t>
-  </si>
-  <si>
     <t>Notabuskjæret</t>
   </si>
   <si>
@@ -799,6 +796,18 @@
   </si>
   <si>
     <t>Flakstadpollen, Flakstad, Øy ved Djupvika (breinessteinan)</t>
+  </si>
+  <si>
+    <t>Nordre Steinskjæret</t>
+  </si>
+  <si>
+    <t>60.268689000296455, 5.219000199094522</t>
+  </si>
+  <si>
+    <t>Bergen</t>
+  </si>
+  <si>
+    <t>Kvinnherad</t>
   </si>
 </sst>
 </file>
@@ -1298,33 +1307,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:V60"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="65" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="36" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="172.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="47.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="172.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1344,13 +1353,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>6</v>
@@ -1392,7 +1401,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -1438,7 +1447,7 @@
       </c>
       <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1484,7 +1493,7 @@
       </c>
       <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>18</v>
       </c>
@@ -1530,7 +1539,7 @@
       </c>
       <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1576,7 +1585,7 @@
       </c>
       <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1622,7 +1631,7 @@
       </c>
       <c r="V6" s="4"/>
     </row>
-    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -1666,7 +1675,7 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1712,7 +1721,7 @@
       </c>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>18</v>
       </c>
@@ -1770,7 +1779,7 @@
       </c>
       <c r="V9" s="26"/>
     </row>
-    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>18</v>
       </c>
@@ -1826,7 +1835,7 @@
       </c>
       <c r="V10" s="26"/>
     </row>
-    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>18</v>
       </c>
@@ -1886,7 +1895,7 @@
       </c>
       <c r="V11" s="5"/>
     </row>
-    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
@@ -1944,7 +1953,7 @@
       </c>
       <c r="V12" s="5"/>
     </row>
-    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>18</v>
       </c>
@@ -2004,287 +2013,291 @@
       </c>
       <c r="V13" s="5"/>
     </row>
-    <row r="14" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="5" t="s">
+    <row r="14" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5" t="s">
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="O14" s="5">
+      <c r="L14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="O14" s="12">
         <v>2</v>
       </c>
-      <c r="P14" s="5">
+      <c r="P14" s="12">
         <v>5</v>
       </c>
-      <c r="Q14" s="5">
+      <c r="Q14" s="12">
         <v>2</v>
       </c>
-      <c r="R14" s="5" t="s">
+      <c r="R14" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="S14" s="5" t="s">
+      <c r="S14" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="T14" s="5" t="s">
+      <c r="T14" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="U14" s="5" t="s">
+      <c r="U14" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="V14" s="5"/>
-    </row>
-    <row r="15" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="7" t="s">
+      <c r="V14" s="12"/>
+    </row>
+    <row r="15" spans="1:22" s="35" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+    </row>
+    <row r="16" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C16" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-    </row>
-    <row r="16" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="14" t="s">
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9"/>
+      <c r="U16" s="9"/>
+      <c r="V16" s="9"/>
+    </row>
+    <row r="17" spans="1:22" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C17" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F17" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15"/>
-    </row>
-    <row r="17" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="15"/>
+      <c r="Q17" s="15"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+      <c r="V17" s="15"/>
+    </row>
+    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C18" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E18" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10" t="s">
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="K17" s="10" t="s">
+      <c r="K18" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L17" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="M17" s="10" t="s">
+      <c r="L18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="M18" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="N17" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="O17" s="10">
+      <c r="N18" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="O18" s="10">
         <v>1</v>
       </c>
-      <c r="P17" s="10">
+      <c r="P18" s="10">
         <v>1</v>
       </c>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="10" t="s">
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="T17" s="10" t="s">
+      <c r="T18" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="U17" s="10" t="s">
+      <c r="U18" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="V17" s="10"/>
-    </row>
-    <row r="18" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="4" t="s">
+      <c r="V18" s="10"/>
+    </row>
+    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4" t="s">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4" t="s">
+      <c r="L19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O18" s="4">
+      <c r="O19" s="4">
         <v>1</v>
       </c>
-      <c r="P18" s="4">
+      <c r="P19" s="4">
         <v>1</v>
       </c>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="4" t="s">
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="T18" s="4" t="s">
+      <c r="T19" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="U18" s="4"/>
-      <c r="V18" s="4"/>
-    </row>
-    <row r="19" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
-      <c r="S19" s="9"/>
-      <c r="T19" s="9"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9"/>
-    </row>
-    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+    </row>
+    <row r="20" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>18</v>
       </c>
@@ -2295,10 +2308,10 @@
         <v>107</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>23</v>
@@ -2322,133 +2335,131 @@
       <c r="U20" s="9"/>
       <c r="V20" s="9"/>
     </row>
-    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="10" t="s">
+    <row r="21" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+    </row>
+    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D22" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E22" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F22" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10" t="s">
+      <c r="G22" s="10"/>
+      <c r="H22" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K22" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L22" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="M21" s="10" t="s">
+      <c r="M22" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="N21" s="10" t="s">
+      <c r="N22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="O21" s="10">
+      <c r="O22" s="10">
         <v>2</v>
       </c>
-      <c r="P21" s="10">
+      <c r="P22" s="10">
         <v>1</v>
       </c>
-      <c r="Q21" s="10">
+      <c r="Q22" s="10">
         <v>2</v>
       </c>
-      <c r="R21" s="10" t="s">
+      <c r="R22" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="S21" s="10" t="s">
+      <c r="S22" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="T21" s="10" t="s">
+      <c r="T22" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="U21" s="10" t="s">
+      <c r="U22" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="V21" s="10"/>
-    </row>
-    <row r="22" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
-      <c r="R22" s="10"/>
-      <c r="S22" s="10"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="10"/>
       <c r="V22" s="10"/>
     </row>
-    <row r="23" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C23" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>118</v>
-      </c>
-      <c r="E23" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="F23" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="L23" s="26" t="s">
-        <v>202</v>
-      </c>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
-      <c r="Q23" s="26"/>
-      <c r="R23" s="26"/>
-      <c r="S23" s="26"/>
-      <c r="T23" s="26"/>
-      <c r="U23" s="26"/>
-      <c r="V23" s="26"/>
-    </row>
-    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10"/>
+    </row>
+    <row r="24" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="28" t="s">
         <v>18</v>
       </c>
@@ -2459,10 +2470,10 @@
         <v>112</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F24" s="28" t="s">
         <v>23</v>
@@ -2488,7 +2499,7 @@
       <c r="U24" s="26"/>
       <c r="V24" s="26"/>
     </row>
-    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="28" t="s">
         <v>18</v>
       </c>
@@ -2499,10 +2510,10 @@
         <v>112</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F25" s="28" t="s">
         <v>23</v>
@@ -2528,94 +2539,74 @@
       <c r="U25" s="26"/>
       <c r="V25" s="26"/>
     </row>
-    <row r="26" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:22" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="L26" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
+      <c r="Q26" s="26"/>
+      <c r="R26" s="26"/>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="26"/>
+      <c r="V26" s="26"/>
+    </row>
+    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="F26" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="K26" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="L26" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="M26" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="N26" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="O26" s="10">
-        <v>1</v>
-      </c>
-      <c r="P26" s="10">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="10">
-        <v>1</v>
-      </c>
-      <c r="R26" s="10"/>
-      <c r="S26" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="T26" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10"/>
-    </row>
-    <row r="27" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>18</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>91</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>124</v>
+        <v>183</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>125</v>
+        <v>248</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="F27" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10" t="s">
+        <v>61</v>
+      </c>
       <c r="H27" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>254</v>
-      </c>
+        <v>249</v>
+      </c>
+      <c r="I27" s="10"/>
       <c r="J27" s="10" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>72</v>
@@ -2624,10 +2615,10 @@
         <v>61</v>
       </c>
       <c r="M27" s="10" t="s">
-        <v>116</v>
+        <v>185</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="O27" s="10">
         <v>1</v>
@@ -2636,119 +2627,125 @@
         <v>1</v>
       </c>
       <c r="Q27" s="10">
-        <v>2</v>
-      </c>
-      <c r="R27" s="10" t="s">
-        <v>81</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R27" s="10"/>
       <c r="S27" s="10" t="s">
         <v>62</v>
       </c>
       <c r="T27" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10"/>
+    </row>
+    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L28" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M28" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="N28" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="O28" s="10">
+        <v>1</v>
+      </c>
+      <c r="P28" s="10">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="10">
+        <v>2</v>
+      </c>
+      <c r="R28" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="S28" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="T28" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="U27" s="13" t="s">
+      <c r="U28" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="V27" s="10"/>
-    </row>
-    <row r="28" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="V28" s="10"/>
+    </row>
+    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C29" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F29" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="I28" s="7">
+      <c r="G29" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="I29" s="7">
         <v>41693935</v>
       </c>
-      <c r="J28" s="8"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
-      <c r="S28" s="9"/>
-      <c r="T28" s="9"/>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9"/>
-    </row>
-    <row r="29" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="I29" s="5">
-        <v>97519210</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="L29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O29" s="5">
-        <v>1</v>
-      </c>
-      <c r="P29" s="5">
-        <v>2</v>
-      </c>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="5"/>
-    </row>
-    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J29" s="8"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="9"/>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
+      <c r="S29" s="9"/>
+      <c r="T29" s="9"/>
+      <c r="U29" s="9"/>
+      <c r="V29" s="9"/>
+    </row>
+    <row r="30" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>18</v>
       </c>
@@ -2759,19 +2756,25 @@
         <v>133</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>136</v>
+        <v>255</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="G30" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="I30" s="5">
+        <v>97519210</v>
+      </c>
       <c r="J30" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>72</v>
@@ -2796,7 +2799,7 @@
       <c r="U30" s="5"/>
       <c r="V30" s="5"/>
     </row>
-    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>18</v>
       </c>
@@ -2807,10 +2810,10 @@
         <v>133</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>23</v>
@@ -2819,7 +2822,7 @@
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K31" s="5" t="s">
         <v>72</v>
@@ -2844,7 +2847,7 @@
       <c r="U31" s="5"/>
       <c r="V31" s="5"/>
     </row>
-    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>18</v>
       </c>
@@ -2855,10 +2858,10 @@
         <v>133</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>143</v>
+        <v>139</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>140</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>23</v>
@@ -2867,7 +2870,7 @@
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>72</v>
@@ -2892,167 +2895,157 @@
       <c r="U32" s="5"/>
       <c r="V32" s="5"/>
     </row>
-    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" s="4" t="s">
+    <row r="33" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="O33" s="5">
+        <v>1</v>
+      </c>
+      <c r="P33" s="5">
+        <v>2</v>
+      </c>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="5"/>
+    </row>
+    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D34" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E34" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4" t="s">
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="K33" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="L33" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4" t="s">
+      <c r="L34" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O34" s="4">
         <v>1</v>
       </c>
-      <c r="P33" s="4">
+      <c r="P34" s="4">
         <v>2</v>
       </c>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="4"/>
-      <c r="T33" s="4"/>
-      <c r="U33" s="4"/>
-      <c r="V33" s="4"/>
-    </row>
-    <row r="34" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" s="12" t="s">
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
+      <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="4"/>
+      <c r="V34" s="4"/>
+    </row>
+    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C35" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D35" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E35" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="F34" s="12" t="s">
+      <c r="F35" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12" t="s">
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="K34" s="12" t="s">
+      <c r="K35" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="L34" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="M34" s="12"/>
-      <c r="N34" s="12" t="s">
+      <c r="L35" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="O34" s="12">
+      <c r="O35" s="12">
         <v>1</v>
       </c>
-      <c r="P34" s="12">
+      <c r="P35" s="12">
         <v>4</v>
       </c>
-      <c r="Q34" s="12"/>
-      <c r="R34" s="12"/>
-      <c r="S34" s="12" t="s">
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="T34" s="12" t="s">
+      <c r="T35" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="U34" s="12" t="s">
+      <c r="U35" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="V34" s="12"/>
-    </row>
-    <row r="35" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="L35" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="M35" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="N35" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="O35" s="4">
-        <v>0.2</v>
-      </c>
-      <c r="P35" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="Q35" s="4">
-        <v>1</v>
-      </c>
-      <c r="R35" s="4"/>
-      <c r="S35" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="T35" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="U35" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="V35" s="4"/>
-    </row>
-    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="V35" s="12"/>
+    </row>
+    <row r="36" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>18</v>
       </c>
@@ -3063,10 +3056,10 @@
         <v>155</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>158</v>
@@ -3075,7 +3068,7 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="K36" s="4" t="s">
         <v>72</v>
@@ -3086,7 +3079,9 @@
       <c r="M36" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="N36" s="4"/>
+      <c r="N36" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="O36" s="4">
         <v>0.2</v>
       </c>
@@ -3108,7 +3103,7 @@
       </c>
       <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>18</v>
       </c>
@@ -3119,10 +3114,10 @@
         <v>155</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>158</v>
@@ -3131,7 +3126,7 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>72</v>
@@ -3142,9 +3137,7 @@
       <c r="M37" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="N37" s="4" t="s">
-        <v>169</v>
-      </c>
+      <c r="N37" s="4"/>
       <c r="O37" s="4">
         <v>0.2</v>
       </c>
@@ -3166,7 +3159,7 @@
       </c>
       <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>18</v>
       </c>
@@ -3177,7 +3170,7 @@
         <v>155</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>167</v>
@@ -3189,7 +3182,7 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="K38" s="4" t="s">
         <v>72</v>
@@ -3201,7 +3194,7 @@
         <v>160</v>
       </c>
       <c r="N38" s="4" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="O38" s="4">
         <v>0.2</v>
@@ -3224,7 +3217,7 @@
       </c>
       <c r="V38" s="4"/>
     </row>
-    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>18</v>
       </c>
@@ -3235,7 +3228,7 @@
         <v>155</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>167</v>
@@ -3247,7 +3240,7 @@
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K39" s="4" t="s">
         <v>72</v>
@@ -3259,7 +3252,7 @@
         <v>160</v>
       </c>
       <c r="N39" s="4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="O39" s="4">
         <v>0.2</v>
@@ -3268,7 +3261,7 @@
         <v>0.5</v>
       </c>
       <c r="Q39" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R39" s="4"/>
       <c r="S39" s="4" t="s">
@@ -3278,96 +3271,102 @@
         <v>75</v>
       </c>
       <c r="U39" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="V39" s="4"/>
+    </row>
+    <row r="40" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L40" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="N40" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="O40" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="P40" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="Q40" s="4">
+        <v>2</v>
+      </c>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="T40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="U40" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="V39" s="4"/>
-    </row>
-    <row r="40" spans="1:22" s="18" customFormat="1" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="V40" s="4"/>
+    </row>
+    <row r="41" spans="1:22" s="18" customFormat="1" ht="15" x14ac:dyDescent="0.35">
+      <c r="A41" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B41" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C41" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D41" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="E40" s="17" t="s">
+      <c r="E41" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="F41" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12" t="s">
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="K40" s="12" t="s">
+      <c r="K41" s="12" t="s">
         <v>72</v>
-      </c>
-      <c r="L40" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="M40" s="12"/>
-      <c r="N40" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="O40" s="12">
-        <v>1</v>
-      </c>
-      <c r="P40" s="12">
-        <v>1</v>
-      </c>
-      <c r="Q40" s="12"/>
-      <c r="R40" s="12"/>
-      <c r="S40" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="T40" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="U40" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="V40" s="12"/>
-    </row>
-    <row r="41" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="36" t="s">
-        <v>62</v>
-      </c>
-      <c r="B41" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="C41" s="36" t="s">
-        <v>187</v>
-      </c>
-      <c r="D41" s="36" t="s">
-        <v>188</v>
-      </c>
-      <c r="E41" s="36"/>
-      <c r="F41" s="36" t="s">
-        <v>189</v>
-      </c>
-      <c r="G41" s="36"/>
-      <c r="H41" s="36"/>
-      <c r="I41" s="36"/>
-      <c r="J41" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="K41" s="12" t="s">
-        <v>25</v>
       </c>
       <c r="L41" s="12" t="s">
         <v>73</v>
       </c>
       <c r="M41" s="12"/>
       <c r="N41" s="12" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="O41" s="12">
         <v>1</v>
@@ -3378,15 +3377,17 @@
       <c r="Q41" s="12"/>
       <c r="R41" s="12"/>
       <c r="S41" s="12" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
       <c r="T41" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="U41" s="12"/>
+        <v>128</v>
+      </c>
+      <c r="U41" s="12" t="s">
+        <v>182</v>
+      </c>
       <c r="V41" s="12"/>
     </row>
-    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="36" t="s">
         <v>62</v>
       </c>
@@ -3397,17 +3398,17 @@
         <v>187</v>
       </c>
       <c r="D42" s="36" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E42" s="36"/>
       <c r="F42" s="36" t="s">
-        <v>73</v>
+        <v>189</v>
       </c>
       <c r="G42" s="36"/>
       <c r="H42" s="36"/>
       <c r="I42" s="36"/>
       <c r="J42" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K42" s="12" t="s">
         <v>25</v>
@@ -3417,7 +3418,7 @@
       </c>
       <c r="M42" s="12"/>
       <c r="N42" s="12" t="s">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="O42" s="12">
         <v>1</v>
@@ -3436,7 +3437,7 @@
       <c r="U42" s="12"/>
       <c r="V42" s="12"/>
     </row>
-    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="36" t="s">
         <v>62</v>
       </c>
@@ -3444,10 +3445,10 @@
         <v>91</v>
       </c>
       <c r="C43" s="36" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D43" s="36" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E43" s="36"/>
       <c r="F43" s="36" t="s">
@@ -3457,7 +3458,7 @@
       <c r="H43" s="36"/>
       <c r="I43" s="36"/>
       <c r="J43" s="12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K43" s="12" t="s">
         <v>25</v>
@@ -3467,7 +3468,7 @@
       </c>
       <c r="M43" s="12"/>
       <c r="N43" s="12" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="O43" s="12">
         <v>1</v>
@@ -3486,63 +3487,57 @@
       <c r="U43" s="12"/>
       <c r="V43" s="12"/>
     </row>
-    <row r="44" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+    <row r="44" spans="1:22" s="18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B44" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="F44" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="K44" s="10" t="s">
+      <c r="B44" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="36" t="s">
+        <v>193</v>
+      </c>
+      <c r="D44" s="36" t="s">
+        <v>194</v>
+      </c>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
+      <c r="J44" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="K44" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="L44" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="M44" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="N44" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="O44" s="10">
+      <c r="L44" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="M44" s="12"/>
+      <c r="N44" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="O44" s="12">
         <v>1</v>
       </c>
-      <c r="P44" s="10">
+      <c r="P44" s="12">
         <v>1</v>
       </c>
-      <c r="Q44" s="10">
-        <v>3</v>
-      </c>
-      <c r="R44" s="10"/>
-      <c r="S44" s="10" t="s">
+      <c r="Q44" s="12"/>
+      <c r="R44" s="12"/>
+      <c r="S44" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="T44" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="U44" s="10"/>
-      <c r="V44" s="10"/>
-    </row>
-    <row r="45" spans="1:22" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="T44" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="U44" s="12"/>
+      <c r="V44" s="12"/>
+    </row>
+    <row r="45" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10" t="s">
         <v>62</v>
       </c>
@@ -3550,63 +3545,55 @@
         <v>154</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G45" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="H45" t="s">
-        <v>242</v>
-      </c>
-      <c r="I45" s="24">
-        <v>48197464</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
       <c r="J45" s="10" t="s">
-        <v>175</v>
+        <v>199</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="M45" s="10" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>73</v>
+        <v>161</v>
       </c>
       <c r="O45" s="10">
         <v>1</v>
       </c>
       <c r="P45" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q45" s="10">
-        <v>4</v>
-      </c>
-      <c r="R45" s="10">
-        <v>2</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="R45" s="10"/>
       <c r="S45" s="10" t="s">
         <v>62</v>
       </c>
       <c r="T45" s="10" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="U45" s="10"/>
       <c r="V45" s="10"/>
     </row>
-    <row r="46" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="10" t="s">
         <v>62</v>
       </c>
@@ -3616,41 +3603,61 @@
       <c r="C46" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D46" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="E46" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="F46" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="G46" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="I46" s="7"/>
-      <c r="J46" s="8"/>
+      <c r="D46" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G46" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="H46" t="s">
+        <v>241</v>
+      </c>
+      <c r="I46" s="24">
+        <v>48197464</v>
+      </c>
+      <c r="J46" s="10" t="s">
+        <v>175</v>
+      </c>
       <c r="K46" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L46" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="M46" s="9"/>
-      <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="9"/>
-      <c r="Q46" s="9"/>
-      <c r="R46" s="9"/>
-      <c r="S46" s="9"/>
-      <c r="T46" s="9"/>
-      <c r="U46" s="9"/>
-      <c r="V46" s="9"/>
-    </row>
-    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L46" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="M46" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="N46" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="O46" s="10">
+        <v>1</v>
+      </c>
+      <c r="P46" s="10">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="10">
+        <v>4</v>
+      </c>
+      <c r="R46" s="10">
+        <v>2</v>
+      </c>
+      <c r="S46" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="T46" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="U46" s="10"/>
+      <c r="V46" s="10"/>
+    </row>
+    <row r="47" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
         <v>62</v>
       </c>
@@ -3660,35 +3667,41 @@
       <c r="C47" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="D47" s="35" t="s">
-        <v>205</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>216</v>
+      <c r="D47" s="34" t="s">
+        <v>204</v>
+      </c>
+      <c r="E47" s="34" t="s">
+        <v>217</v>
       </c>
       <c r="F47" s="34" t="s">
         <v>73</v>
       </c>
       <c r="G47" s="34" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>243</v>
-      </c>
+        <v>247</v>
+      </c>
+      <c r="I47" s="7"/>
+      <c r="J47" s="8"/>
       <c r="K47" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="L47" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="N47" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="L47" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="9"/>
+      <c r="R47" s="9"/>
+      <c r="S47" s="9"/>
+      <c r="T47" s="9"/>
+      <c r="U47" s="9"/>
+      <c r="V47" s="9"/>
+    </row>
+    <row r="48" spans="1:22" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>62</v>
       </c>
@@ -3699,72 +3712,72 @@
         <v>203</v>
       </c>
       <c r="D48" s="35" t="s">
-        <v>206</v>
-      </c>
-      <c r="E48" s="34" t="s">
-        <v>218</v>
+        <v>205</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>216</v>
       </c>
       <c r="F48" s="34" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="G48" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="H48" t="s">
-        <v>247</v>
-      </c>
-      <c r="I48" s="7">
-        <v>91389435</v>
+      <c r="H48" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="I48" s="7" t="s">
+        <v>242</v>
       </c>
       <c r="K48" s="10" t="s">
         <v>72</v>
       </c>
       <c r="L48" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N48" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D49" s="35" t="s">
+        <v>206</v>
+      </c>
+      <c r="E49" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="F49" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="G49" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="H49" t="s">
+        <v>246</v>
+      </c>
+      <c r="I49" s="7">
+        <v>91389435</v>
+      </c>
+      <c r="K49" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L49" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="N48" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="B49" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>207</v>
-      </c>
-      <c r="D49" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="E49" s="26" t="s">
-        <v>215</v>
-      </c>
-      <c r="F49" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="G49" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="H49" s="28" t="s">
-        <v>240</v>
-      </c>
-      <c r="I49" s="28">
-        <v>94123558</v>
-      </c>
-      <c r="K49" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="L49" s="27" t="s">
-        <v>202</v>
-      </c>
-      <c r="N49" s="26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="N49" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="26" t="s">
         <v>62</v>
       </c>
@@ -3775,10 +3788,10 @@
         <v>207</v>
       </c>
       <c r="D50" s="27" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E50" s="26" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F50" s="28" t="s">
         <v>61</v>
@@ -3786,8 +3799,12 @@
       <c r="G50" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="H50" s="28"/>
-      <c r="I50" s="28"/>
+      <c r="H50" s="28" t="s">
+        <v>239</v>
+      </c>
+      <c r="I50" s="28">
+        <v>94123558</v>
+      </c>
       <c r="K50" s="26" t="s">
         <v>25</v>
       </c>
@@ -3798,45 +3815,41 @@
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10" t="s">
+    <row r="51" spans="1:14" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B51" s="10" t="s">
+      <c r="B51" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="D51" s="35" t="s">
-        <v>209</v>
-      </c>
-      <c r="E51" s="35" t="s">
-        <v>211</v>
-      </c>
-      <c r="F51" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="G51" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="H51" t="s">
-        <v>245</v>
-      </c>
-      <c r="I51" t="s">
-        <v>246</v>
-      </c>
-      <c r="K51" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="N51" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D51" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="E51" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="F51" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="G51" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="H51" s="28"/>
+      <c r="I51" s="28"/>
+      <c r="K51" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="L51" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="N51" s="26" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
         <v>62</v>
       </c>
@@ -3847,19 +3860,23 @@
         <v>207</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>210</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>212</v>
+        <v>209</v>
+      </c>
+      <c r="E52" s="35" t="s">
+        <v>211</v>
       </c>
       <c r="F52" s="34" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="G52" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="H52" s="7"/>
-      <c r="I52" s="7"/>
+        <v>61</v>
+      </c>
+      <c r="H52" t="s">
+        <v>244</v>
+      </c>
+      <c r="I52" t="s">
+        <v>245</v>
+      </c>
       <c r="K52" s="10" t="s">
         <v>72</v>
       </c>
@@ -3870,68 +3887,91 @@
         <v>73</v>
       </c>
     </row>
-    <row r="53" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="B53" s="26" t="s">
+    <row r="53" spans="1:14" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D53" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="F53" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="G53" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+      <c r="K53" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="N53" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="D53" s="30" t="s">
+      <c r="C54" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="D54" s="30" t="s">
         <v>220</v>
       </c>
-      <c r="E53" s="29" t="s">
+      <c r="E54" s="29" t="s">
         <v>221</v>
       </c>
-      <c r="F53" s="31" t="s">
-        <v>61</v>
-      </c>
-      <c r="G53" s="32"/>
-      <c r="H53" s="32"/>
-      <c r="I53" s="32"/>
-      <c r="K53" s="33" t="s">
+      <c r="F54" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="G54" s="32"/>
+      <c r="H54" s="32"/>
+      <c r="I54" s="32"/>
+      <c r="K54" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="L53" s="30" t="s">
+      <c r="L54" s="30" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="E54" t="s">
-        <v>223</v>
-      </c>
-      <c r="F54" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="K54" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="L54" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>56</v>
       </c>
+      <c r="C55" t="s">
+        <v>259</v>
+      </c>
       <c r="D55" s="19" t="s">
-        <v>224</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="E55" t="s">
+        <v>223</v>
+      </c>
+      <c r="F55" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G55" s="23"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
       <c r="K55" s="20" t="s">
         <v>72</v>
       </c>
@@ -3939,7 +3979,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>18</v>
       </c>
@@ -3947,22 +3987,19 @@
         <v>56</v>
       </c>
       <c r="C56" t="s">
-        <v>226</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="E56" t="s">
-        <v>227</v>
+        <v>259</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>224</v>
       </c>
       <c r="K56" s="20" t="s">
         <v>72</v>
       </c>
       <c r="L56" s="19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>18</v>
       </c>
@@ -3970,22 +4007,22 @@
         <v>56</v>
       </c>
       <c r="C57" t="s">
-        <v>230</v>
-      </c>
-      <c r="D57" t="s">
-        <v>228</v>
+        <v>226</v>
+      </c>
+      <c r="D57" s="22" t="s">
+        <v>225</v>
       </c>
       <c r="E57" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="K57" s="20" t="s">
         <v>72</v>
       </c>
       <c r="L57" s="19" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>18</v>
       </c>
@@ -3993,13 +4030,13 @@
         <v>56</v>
       </c>
       <c r="C58" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D58" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E58" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="K58" s="20" t="s">
         <v>72</v>
@@ -4008,7 +4045,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>18</v>
       </c>
@@ -4016,16 +4053,13 @@
         <v>56</v>
       </c>
       <c r="C59" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D59" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E59" t="s">
-        <v>236</v>
-      </c>
-      <c r="F59" t="s">
-        <v>73</v>
+        <v>232</v>
       </c>
       <c r="K59" s="20" t="s">
         <v>72</v>
@@ -4034,8 +4068,34 @@
         <v>61</v>
       </c>
     </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60" t="s">
+        <v>258</v>
+      </c>
+      <c r="D60" t="s">
+        <v>234</v>
+      </c>
+      <c r="E60" t="s">
+        <v>235</v>
+      </c>
+      <c r="F60" t="s">
+        <v>73</v>
+      </c>
+      <c r="K60" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="L60" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V59" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V60" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>